<commit_message>
feat: fiche PDF biosimilaires (poster facon Teva) + prix PPHT/net IP
- generate_biosim_pdf.js : poster brande Integral, 2 versions
  * pharmacien (PPHT + abandon %, sans net IP) -> telechargeable depuis le CRM
  * interne (PPHT + net IP + confidentiel) -> local, gitignore (jamais publie)
- robot : PPHT officiel (ppht-data.js) + net IP calcule (barème abandon) +
  pack standard par molecule (prix comparable marque a marque)
- page CRM : bouton telechargement de la fiche PDF pharmacien
- cache-busting -> 20260710e

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/base-biosimilaires.xlsx
+++ b/base-biosimilaires.xlsx
@@ -2244,10 +2244,10 @@
       </c>
       <c r="P3" s="5" t="inlineStr"/>
       <c r="Q3" s="5" t="n">
-        <v>354.74</v>
+        <v>394.08</v>
       </c>
       <c r="R3" s="5" t="n">
-        <v>340.94</v>
+        <v>378.75</v>
       </c>
       <c r="S3" s="5" t="n">
         <v>16</v>
@@ -2335,10 +2335,10 @@
         <v>13</v>
       </c>
       <c r="Q4" s="2" t="n">
-        <v>197.36</v>
+        <v>354.74</v>
       </c>
       <c r="R4" s="2" t="n">
-        <v>189.68</v>
+        <v>340.94</v>
       </c>
       <c r="S4" s="2" t="n">
         <v>10</v>
@@ -2585,8 +2585,12 @@
       <c r="P7" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="Q7" s="2" t="inlineStr"/>
-      <c r="R7" s="2" t="inlineStr"/>
+      <c r="Q7" s="2" t="n">
+        <v>354.74</v>
+      </c>
+      <c r="R7" s="2" t="n">
+        <v>340.94</v>
+      </c>
       <c r="S7" s="2" t="n">
         <v>6</v>
       </c>
@@ -2660,8 +2664,12 @@
       </c>
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr"/>
-      <c r="Q8" s="2" t="inlineStr"/>
-      <c r="R8" s="2" t="inlineStr"/>
+      <c r="Q8" s="2" t="n">
+        <v>354.74</v>
+      </c>
+      <c r="R8" s="2" t="n">
+        <v>340.94</v>
+      </c>
       <c r="S8" s="2" t="n">
         <v>2</v>
       </c>
@@ -2735,8 +2743,12 @@
       </c>
       <c r="O9" s="2" t="inlineStr"/>
       <c r="P9" s="2" t="inlineStr"/>
-      <c r="Q9" s="2" t="inlineStr"/>
-      <c r="R9" s="2" t="inlineStr"/>
+      <c r="Q9" s="2" t="n">
+        <v>354.74</v>
+      </c>
+      <c r="R9" s="2" t="n">
+        <v>340.94</v>
+      </c>
       <c r="S9" s="2" t="inlineStr"/>
       <c r="T9" s="2" t="inlineStr"/>
       <c r="U9" s="2" t="inlineStr">
@@ -2897,8 +2909,12 @@
       <c r="P11" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="Q11" s="2" t="inlineStr"/>
-      <c r="R11" s="2" t="inlineStr"/>
+      <c r="Q11" s="2" t="n">
+        <v>354.74</v>
+      </c>
+      <c r="R11" s="2" t="n">
+        <v>340.94</v>
+      </c>
       <c r="S11" s="2" t="n">
         <v>1</v>
       </c>
@@ -2978,8 +2994,12 @@
       <c r="P12" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="Q12" s="2" t="inlineStr"/>
-      <c r="R12" s="2" t="inlineStr"/>
+      <c r="Q12" s="2" t="n">
+        <v>354.74</v>
+      </c>
+      <c r="R12" s="2" t="n">
+        <v>340.94</v>
+      </c>
       <c r="S12" s="2" t="n">
         <v>2</v>
       </c>
@@ -3061,8 +3081,12 @@
       <c r="P13" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="Q13" s="5" t="inlineStr"/>
-      <c r="R13" s="5" t="inlineStr"/>
+      <c r="Q13" s="5" t="n">
+        <v>441.16</v>
+      </c>
+      <c r="R13" s="5" t="n">
+        <v>424</v>
+      </c>
       <c r="S13" s="5" t="n">
         <v>5</v>
       </c>
@@ -3223,8 +3247,12 @@
       <c r="P15" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="Q15" s="2" t="inlineStr"/>
-      <c r="R15" s="2" t="inlineStr"/>
+      <c r="Q15" s="2" t="n">
+        <v>441.16</v>
+      </c>
+      <c r="R15" s="2" t="n">
+        <v>424</v>
+      </c>
       <c r="S15" s="2" t="n">
         <v>3</v>
       </c>
@@ -3696,8 +3724,12 @@
       <c r="P22" s="5" t="n">
         <v>17</v>
       </c>
-      <c r="Q22" s="5" t="inlineStr"/>
-      <c r="R22" s="5" t="inlineStr"/>
+      <c r="Q22" s="5" t="n">
+        <v>477.98</v>
+      </c>
+      <c r="R22" s="5" t="n">
+        <v>458.48</v>
+      </c>
       <c r="S22" s="5" t="n">
         <v>11</v>
       </c>
@@ -3883,8 +3915,12 @@
       </c>
       <c r="O25" s="5" t="inlineStr"/>
       <c r="P25" s="5" t="inlineStr"/>
-      <c r="Q25" s="5" t="inlineStr"/>
-      <c r="R25" s="5" t="inlineStr"/>
+      <c r="Q25" s="5" t="n">
+        <v>1393.18</v>
+      </c>
+      <c r="R25" s="5" t="n">
+        <v>1373.68</v>
+      </c>
       <c r="S25" s="5" t="n">
         <v>8</v>
       </c>
@@ -4045,8 +4081,12 @@
       </c>
       <c r="O27" s="2" t="inlineStr"/>
       <c r="P27" s="2" t="inlineStr"/>
-      <c r="Q27" s="2" t="inlineStr"/>
-      <c r="R27" s="2" t="inlineStr"/>
+      <c r="Q27" s="2" t="n">
+        <v>1053.17</v>
+      </c>
+      <c r="R27" s="2" t="n">
+        <v>1033.67</v>
+      </c>
       <c r="S27" s="2" t="inlineStr"/>
       <c r="T27" s="2" t="inlineStr">
         <is>
@@ -4122,8 +4162,12 @@
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
-      <c r="Q28" s="2" t="inlineStr"/>
-      <c r="R28" s="2" t="inlineStr"/>
+      <c r="Q28" s="2" t="n">
+        <v>1053.17</v>
+      </c>
+      <c r="R28" s="2" t="n">
+        <v>1033.67</v>
+      </c>
       <c r="S28" s="2" t="inlineStr"/>
       <c r="T28" s="2" t="inlineStr">
         <is>
@@ -4197,8 +4241,12 @@
       <c r="P29" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="Q29" s="2" t="inlineStr"/>
-      <c r="R29" s="2" t="inlineStr"/>
+      <c r="Q29" s="2" t="n">
+        <v>1053.17</v>
+      </c>
+      <c r="R29" s="2" t="n">
+        <v>1033.67</v>
+      </c>
       <c r="S29" s="2" t="inlineStr"/>
       <c r="T29" s="2" t="inlineStr">
         <is>
@@ -4272,8 +4320,12 @@
       <c r="P30" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="Q30" s="2" t="inlineStr"/>
-      <c r="R30" s="2" t="inlineStr"/>
+      <c r="Q30" s="2" t="n">
+        <v>1053.17</v>
+      </c>
+      <c r="R30" s="2" t="n">
+        <v>1033.67</v>
+      </c>
       <c r="S30" s="2" t="inlineStr"/>
       <c r="T30" s="2" t="inlineStr">
         <is>
@@ -4457,8 +4509,12 @@
       </c>
       <c r="O33" s="5" t="inlineStr"/>
       <c r="P33" s="5" t="inlineStr"/>
-      <c r="Q33" s="5" t="inlineStr"/>
-      <c r="R33" s="5" t="inlineStr"/>
+      <c r="Q33" s="5" t="n">
+        <v>534.39</v>
+      </c>
+      <c r="R33" s="5" t="n">
+        <v>514.89</v>
+      </c>
       <c r="S33" s="5" t="n">
         <v>7</v>
       </c>
@@ -4532,8 +4588,12 @@
       </c>
       <c r="O34" s="2" t="inlineStr"/>
       <c r="P34" s="2" t="inlineStr"/>
-      <c r="Q34" s="2" t="inlineStr"/>
-      <c r="R34" s="2" t="inlineStr"/>
+      <c r="Q34" s="2" t="n">
+        <v>449.93</v>
+      </c>
+      <c r="R34" s="2" t="n">
+        <v>432.43</v>
+      </c>
       <c r="S34" s="2" t="n">
         <v>1</v>
       </c>
@@ -4605,8 +4665,12 @@
       <c r="P35" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="Q35" s="2" t="inlineStr"/>
-      <c r="R35" s="2" t="inlineStr"/>
+      <c r="Q35" s="2" t="n">
+        <v>112.95</v>
+      </c>
+      <c r="R35" s="2" t="n">
+        <v>108.56</v>
+      </c>
       <c r="S35" s="2" t="inlineStr"/>
       <c r="T35" s="2" t="inlineStr">
         <is>
@@ -6347,8 +6411,12 @@
       <c r="P65" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="Q65" s="5" t="inlineStr"/>
-      <c r="R65" s="5" t="inlineStr"/>
+      <c r="Q65" s="5" t="n">
+        <v>54.62</v>
+      </c>
+      <c r="R65" s="5" t="n">
+        <v>52.5</v>
+      </c>
       <c r="S65" s="5" t="n">
         <v>1</v>
       </c>
@@ -6519,8 +6587,12 @@
       <c r="P67" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="Q67" s="2" t="inlineStr"/>
-      <c r="R67" s="2" t="inlineStr"/>
+      <c r="Q67" s="2" t="n">
+        <v>54.62</v>
+      </c>
+      <c r="R67" s="2" t="n">
+        <v>52.5</v>
+      </c>
       <c r="S67" s="2" t="n">
         <v>3</v>
       </c>
@@ -6602,8 +6674,12 @@
       </c>
       <c r="O68" s="2" t="inlineStr"/>
       <c r="P68" s="2" t="inlineStr"/>
-      <c r="Q68" s="2" t="inlineStr"/>
-      <c r="R68" s="2" t="inlineStr"/>
+      <c r="Q68" s="2" t="n">
+        <v>54.62</v>
+      </c>
+      <c r="R68" s="2" t="n">
+        <v>52.5</v>
+      </c>
       <c r="S68" s="2" t="n">
         <v>5</v>
       </c>
@@ -6675,8 +6751,12 @@
       <c r="P69" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="Q69" s="2" t="inlineStr"/>
-      <c r="R69" s="2" t="inlineStr"/>
+      <c r="Q69" s="2" t="n">
+        <v>54.62</v>
+      </c>
+      <c r="R69" s="2" t="n">
+        <v>52.5</v>
+      </c>
       <c r="S69" s="2" t="n">
         <v>7</v>
       </c>
@@ -6949,8 +7029,12 @@
       </c>
       <c r="O73" s="5" t="inlineStr"/>
       <c r="P73" s="5" t="inlineStr"/>
-      <c r="Q73" s="5" t="inlineStr"/>
-      <c r="R73" s="5" t="inlineStr"/>
+      <c r="Q73" s="5" t="n">
+        <v>363.4</v>
+      </c>
+      <c r="R73" s="5" t="n">
+        <v>349.26</v>
+      </c>
       <c r="S73" s="5" t="n">
         <v>1</v>
       </c>
@@ -7028,8 +7112,12 @@
       </c>
       <c r="O74" s="2" t="inlineStr"/>
       <c r="P74" s="2" t="inlineStr"/>
-      <c r="Q74" s="2" t="inlineStr"/>
-      <c r="R74" s="2" t="inlineStr"/>
+      <c r="Q74" s="2" t="n">
+        <v>363.4</v>
+      </c>
+      <c r="R74" s="2" t="n">
+        <v>349.26</v>
+      </c>
       <c r="S74" s="2" t="n">
         <v>4</v>
       </c>
@@ -7105,8 +7193,12 @@
       <c r="P75" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="Q75" s="2" t="inlineStr"/>
-      <c r="R75" s="2" t="inlineStr"/>
+      <c r="Q75" s="2" t="n">
+        <v>363.39</v>
+      </c>
+      <c r="R75" s="2" t="n">
+        <v>349.25</v>
+      </c>
       <c r="S75" s="2" t="n">
         <v>2</v>
       </c>
@@ -7182,8 +7274,12 @@
       <c r="P76" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="Q76" s="2" t="inlineStr"/>
-      <c r="R76" s="2" t="inlineStr"/>
+      <c r="Q76" s="2" t="n">
+        <v>363.4</v>
+      </c>
+      <c r="R76" s="2" t="n">
+        <v>349.26</v>
+      </c>
       <c r="S76" s="2" t="n">
         <v>2</v>
       </c>
@@ -7263,8 +7359,12 @@
       <c r="P77" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="Q77" s="2" t="inlineStr"/>
-      <c r="R77" s="2" t="inlineStr"/>
+      <c r="Q77" s="2" t="n">
+        <v>363.4</v>
+      </c>
+      <c r="R77" s="2" t="n">
+        <v>349.26</v>
+      </c>
       <c r="S77" s="2" t="n">
         <v>2</v>
       </c>
@@ -7431,8 +7531,12 @@
       <c r="P79" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="Q79" s="2" t="inlineStr"/>
-      <c r="R79" s="2" t="inlineStr"/>
+      <c r="Q79" s="2" t="n">
+        <v>363.4</v>
+      </c>
+      <c r="R79" s="2" t="n">
+        <v>349.26</v>
+      </c>
       <c r="S79" s="2" t="inlineStr"/>
       <c r="T79" s="2" t="inlineStr">
         <is>
@@ -7504,8 +7608,12 @@
       </c>
       <c r="O80" s="2" t="inlineStr"/>
       <c r="P80" s="2" t="inlineStr"/>
-      <c r="Q80" s="2" t="inlineStr"/>
-      <c r="R80" s="2" t="inlineStr"/>
+      <c r="Q80" s="2" t="n">
+        <v>363.4</v>
+      </c>
+      <c r="R80" s="2" t="n">
+        <v>349.26</v>
+      </c>
       <c r="S80" s="2" t="n">
         <v>3</v>
       </c>
@@ -7587,8 +7695,12 @@
       </c>
       <c r="O81" s="2" t="inlineStr"/>
       <c r="P81" s="2" t="inlineStr"/>
-      <c r="Q81" s="2" t="inlineStr"/>
-      <c r="R81" s="2" t="inlineStr"/>
+      <c r="Q81" s="2" t="n">
+        <v>363.4</v>
+      </c>
+      <c r="R81" s="2" t="n">
+        <v>349.26</v>
+      </c>
       <c r="S81" s="2" t="n">
         <v>1</v>
       </c>
@@ -8305,8 +8417,12 @@
       <c r="P91" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="Q91" s="2" t="inlineStr"/>
-      <c r="R91" s="2" t="inlineStr"/>
+      <c r="Q91" s="2" t="n">
+        <v>32.63</v>
+      </c>
+      <c r="R91" s="2" t="n">
+        <v>31.36</v>
+      </c>
       <c r="S91" s="2" t="inlineStr"/>
       <c r="T91" s="2" t="inlineStr">
         <is>
@@ -8379,10 +8495,10 @@
       </c>
       <c r="P92" s="5" t="inlineStr"/>
       <c r="Q92" s="5" t="n">
-        <v>11.78</v>
+        <v>20.39</v>
       </c>
       <c r="R92" s="5" t="n">
-        <v>11.32</v>
+        <v>19.59</v>
       </c>
       <c r="S92" s="5" t="n">
         <v>186</v>
@@ -8578,10 +8694,10 @@
         <v>31</v>
       </c>
       <c r="Q95" s="5" t="n">
-        <v>13.14</v>
+        <v>25.97</v>
       </c>
       <c r="R95" s="5" t="n">
-        <v>12.63</v>
+        <v>24.96</v>
       </c>
       <c r="S95" s="5" t="n">
         <v>97</v>
@@ -8794,8 +8910,12 @@
       <c r="P98" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="Q98" s="2" t="inlineStr"/>
-      <c r="R98" s="2" t="inlineStr"/>
+      <c r="Q98" s="2" t="n">
+        <v>288.45</v>
+      </c>
+      <c r="R98" s="2" t="n">
+        <v>277.23</v>
+      </c>
       <c r="S98" s="2" t="n">
         <v>1</v>
       </c>
@@ -8877,8 +8997,12 @@
       </c>
       <c r="O99" s="2" t="inlineStr"/>
       <c r="P99" s="2" t="inlineStr"/>
-      <c r="Q99" s="2" t="inlineStr"/>
-      <c r="R99" s="2" t="inlineStr"/>
+      <c r="Q99" s="2" t="n">
+        <v>288.45</v>
+      </c>
+      <c r="R99" s="2" t="n">
+        <v>277.23</v>
+      </c>
       <c r="S99" s="2" t="n">
         <v>2</v>
       </c>
@@ -8960,8 +9084,12 @@
       </c>
       <c r="O100" s="2" t="inlineStr"/>
       <c r="P100" s="2" t="inlineStr"/>
-      <c r="Q100" s="2" t="inlineStr"/>
-      <c r="R100" s="2" t="inlineStr"/>
+      <c r="Q100" s="2" t="n">
+        <v>288.45</v>
+      </c>
+      <c r="R100" s="2" t="n">
+        <v>277.23</v>
+      </c>
       <c r="S100" s="2" t="inlineStr"/>
       <c r="T100" s="2" t="inlineStr">
         <is>
@@ -9031,8 +9159,12 @@
       <c r="P101" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="Q101" s="2" t="inlineStr"/>
-      <c r="R101" s="2" t="inlineStr"/>
+      <c r="Q101" s="2" t="n">
+        <v>288.45</v>
+      </c>
+      <c r="R101" s="2" t="n">
+        <v>277.23</v>
+      </c>
       <c r="S101" s="2" t="inlineStr"/>
       <c r="T101" s="2" t="inlineStr">
         <is>
@@ -9199,8 +9331,12 @@
       <c r="P103" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="Q103" s="2" t="inlineStr"/>
-      <c r="R103" s="2" t="inlineStr"/>
+      <c r="Q103" s="2" t="n">
+        <v>227.38</v>
+      </c>
+      <c r="R103" s="2" t="n">
+        <v>218.53</v>
+      </c>
       <c r="S103" s="2" t="n">
         <v>1</v>
       </c>
@@ -9443,8 +9579,12 @@
       <c r="P107" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="Q107" s="2" t="inlineStr"/>
-      <c r="R107" s="2" t="inlineStr"/>
+      <c r="Q107" s="2" t="n">
+        <v>227.38</v>
+      </c>
+      <c r="R107" s="2" t="n">
+        <v>218.53</v>
+      </c>
       <c r="S107" s="2" t="inlineStr"/>
       <c r="T107" s="2" t="inlineStr">
         <is>
@@ -9724,9 +9864,11 @@
         <v>18</v>
       </c>
       <c r="Q111" s="2" t="n">
-        <v>41.2</v>
-      </c>
-      <c r="R111" s="2" t="inlineStr"/>
+        <v>185.33</v>
+      </c>
+      <c r="R111" s="2" t="n">
+        <v>178.12</v>
+      </c>
       <c r="S111" s="2" t="n">
         <v>3</v>
       </c>
@@ -9800,8 +9942,12 @@
       </c>
       <c r="O112" s="2" t="inlineStr"/>
       <c r="P112" s="2" t="inlineStr"/>
-      <c r="Q112" s="2" t="inlineStr"/>
-      <c r="R112" s="2" t="inlineStr"/>
+      <c r="Q112" s="2" t="n">
+        <v>185.33</v>
+      </c>
+      <c r="R112" s="2" t="n">
+        <v>178.12</v>
+      </c>
       <c r="S112" s="2" t="n">
         <v>1</v>
       </c>
@@ -9875,8 +10021,12 @@
       </c>
       <c r="O113" s="2" t="inlineStr"/>
       <c r="P113" s="2" t="inlineStr"/>
-      <c r="Q113" s="2" t="inlineStr"/>
-      <c r="R113" s="2" t="inlineStr"/>
+      <c r="Q113" s="2" t="n">
+        <v>185.33</v>
+      </c>
+      <c r="R113" s="2" t="n">
+        <v>178.12</v>
+      </c>
       <c r="S113" s="2" t="n">
         <v>1</v>
       </c>
@@ -9950,8 +10100,12 @@
       </c>
       <c r="O114" s="2" t="inlineStr"/>
       <c r="P114" s="2" t="inlineStr"/>
-      <c r="Q114" s="2" t="inlineStr"/>
-      <c r="R114" s="2" t="inlineStr"/>
+      <c r="Q114" s="2" t="n">
+        <v>185.96</v>
+      </c>
+      <c r="R114" s="2" t="n">
+        <v>178.73</v>
+      </c>
       <c r="S114" s="2" t="n">
         <v>1</v>
       </c>
@@ -10163,8 +10317,12 @@
       <c r="N117" s="2" t="inlineStr"/>
       <c r="O117" s="2" t="inlineStr"/>
       <c r="P117" s="2" t="inlineStr"/>
-      <c r="Q117" s="2" t="inlineStr"/>
-      <c r="R117" s="2" t="inlineStr"/>
+      <c r="Q117" s="2" t="n">
+        <v>143.71</v>
+      </c>
+      <c r="R117" s="2" t="n">
+        <v>138.12</v>
+      </c>
       <c r="S117" s="2" t="inlineStr"/>
       <c r="T117" s="2" t="inlineStr">
         <is>
@@ -10234,8 +10392,12 @@
       <c r="P118" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="Q118" s="2" t="inlineStr"/>
-      <c r="R118" s="2" t="inlineStr"/>
+      <c r="Q118" s="2" t="n">
+        <v>143.71</v>
+      </c>
+      <c r="R118" s="2" t="n">
+        <v>138.12</v>
+      </c>
       <c r="S118" s="2" t="inlineStr"/>
       <c r="T118" s="2" t="inlineStr">
         <is>
@@ -10305,8 +10467,12 @@
       <c r="P119" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="Q119" s="2" t="inlineStr"/>
-      <c r="R119" s="2" t="inlineStr"/>
+      <c r="Q119" s="2" t="n">
+        <v>143.71</v>
+      </c>
+      <c r="R119" s="2" t="n">
+        <v>138.12</v>
+      </c>
       <c r="S119" s="2" t="inlineStr"/>
       <c r="T119" s="2" t="inlineStr">
         <is>
@@ -10490,8 +10656,12 @@
       <c r="P122" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="Q122" s="2" t="inlineStr"/>
-      <c r="R122" s="2" t="inlineStr"/>
+      <c r="Q122" s="2" t="n">
+        <v>143.71</v>
+      </c>
+      <c r="R122" s="2" t="n">
+        <v>138.12</v>
+      </c>
       <c r="S122" s="2" t="inlineStr"/>
       <c r="T122" s="2" t="inlineStr">
         <is>
@@ -10742,8 +10912,12 @@
       <c r="P126" s="5" t="n">
         <v>126</v>
       </c>
-      <c r="Q126" s="5" t="inlineStr"/>
-      <c r="R126" s="5" t="inlineStr"/>
+      <c r="Q126" s="5" t="n">
+        <v>23.34</v>
+      </c>
+      <c r="R126" s="5" t="n">
+        <v>22.43</v>
+      </c>
       <c r="S126" s="5" t="n">
         <v>63</v>
       </c>
@@ -10823,8 +10997,12 @@
       <c r="P127" s="2" t="n">
         <v>38</v>
       </c>
-      <c r="Q127" s="2" t="inlineStr"/>
-      <c r="R127" s="2" t="inlineStr"/>
+      <c r="Q127" s="2" t="n">
+        <v>23.34</v>
+      </c>
+      <c r="R127" s="2" t="n">
+        <v>22.43</v>
+      </c>
       <c r="S127" s="2" t="n">
         <v>56</v>
       </c>
@@ -11012,8 +11190,12 @@
       </c>
       <c r="O130" s="2" t="inlineStr"/>
       <c r="P130" s="2" t="inlineStr"/>
-      <c r="Q130" s="2" t="inlineStr"/>
-      <c r="R130" s="2" t="inlineStr"/>
+      <c r="Q130" s="2" t="n">
+        <v>44.85</v>
+      </c>
+      <c r="R130" s="2" t="n">
+        <v>43.11</v>
+      </c>
       <c r="S130" s="2" t="inlineStr"/>
       <c r="T130" s="2" t="inlineStr">
         <is>
@@ -11302,8 +11484,12 @@
       <c r="P134" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="Q134" s="2" t="inlineStr"/>
-      <c r="R134" s="2" t="inlineStr"/>
+      <c r="Q134" s="2" t="n">
+        <v>149.79</v>
+      </c>
+      <c r="R134" s="2" t="n">
+        <v>143.96</v>
+      </c>
       <c r="S134" s="2" t="n">
         <v>4</v>
       </c>
@@ -11379,8 +11565,12 @@
       <c r="P135" s="2" t="n">
         <v>122</v>
       </c>
-      <c r="Q135" s="2" t="inlineStr"/>
-      <c r="R135" s="2" t="inlineStr"/>
+      <c r="Q135" s="2" t="n">
+        <v>13.04</v>
+      </c>
+      <c r="R135" s="2" t="n">
+        <v>12.53</v>
+      </c>
       <c r="S135" s="2" t="n">
         <v>26</v>
       </c>

</xml_diff>